<commit_message>
Update DateBase/orders/Dang Nguyen 195_2026-6-27.xlsx
</commit_message>
<xml_diff>
--- a/DateBase/orders/Dang Nguyen 195_2026-6-27.xlsx
+++ b/DateBase/orders/Dang Nguyen 195_2026-6-27.xlsx
@@ -771,6 +771,9 @@
       <c r="C41" t="str">
         <v>616_康乃馨紫精灵_Purple Elves_undefined_20stems</v>
       </c>
+      <c r="F41" t="str">
+        <v>5</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
@@ -829,7 +832,7 @@
         <v>0.00</v>
       </c>
       <c r="G2" t="str">
-        <v>0310108610197778158303030205558515510555556451055550</v>
+        <v>0310108610197778158303030205558515510555556451055555</v>
       </c>
     </row>
   </sheetData>

</xml_diff>